<commit_message>
chore(data): sync FEB data 2026-03-27 19:18
</commit_message>
<xml_diff>
--- a/data/3FEB_25_26/teams_25_26_3FEB.xlsx
+++ b/data/3FEB_25_26/teams_25_26_3FEB.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD15"/>
+  <dimension ref="A1:CD15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -579,6 +579,266 @@
           <t>PJ</t>
         </is>
       </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_MINUTOS JUGADOS</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_T2 CONVERTIDO</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_T2 INTENTADO</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_T3 CONVERTIDO</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_T3 INTENTADO</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_TL CONVERTIDOS</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_TL INTENTADOS</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_REB OFFENSIVO</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_REB DEFENSIVO</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_ASISTENCIAS</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_RECUPEROS</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_PERDIDAS</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_FaltasCOMETIDAS</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_FaltasRECIBIDAS</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_TAPONES</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_PLAYS</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_POSS</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_PPP</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_PPP OPP</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_OFFRTG</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_DEFRTG</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_NETRTG</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_%OREB</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_%DREB</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_%REB</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>LOCAL_PJ</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_MINUTOS JUGADOS</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_T2 CONVERTIDO</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_T2 INTENTADO</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_T3 CONVERTIDO</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_T3 INTENTADO</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_TL CONVERTIDOS</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_TL INTENTADOS</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_REB OFFENSIVO</t>
+        </is>
+      </c>
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_REB DEFENSIVO</t>
+        </is>
+      </c>
+      <c r="BN1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_ASISTENCIAS</t>
+        </is>
+      </c>
+      <c r="BO1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_RECUPEROS</t>
+        </is>
+      </c>
+      <c r="BP1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_PERDIDAS</t>
+        </is>
+      </c>
+      <c r="BQ1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_FaltasCOMETIDAS</t>
+        </is>
+      </c>
+      <c r="BR1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_FaltasRECIBIDAS</t>
+        </is>
+      </c>
+      <c r="BS1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_TAPONES</t>
+        </is>
+      </c>
+      <c r="BT1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_PLAYS</t>
+        </is>
+      </c>
+      <c r="BU1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_POSS</t>
+        </is>
+      </c>
+      <c r="BV1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_PPP</t>
+        </is>
+      </c>
+      <c r="BW1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_PPP OPP</t>
+        </is>
+      </c>
+      <c r="BX1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_OFFRTG</t>
+        </is>
+      </c>
+      <c r="BY1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_DEFRTG</t>
+        </is>
+      </c>
+      <c r="BZ1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_NETRTG</t>
+        </is>
+      </c>
+      <c r="CA1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_%OREB</t>
+        </is>
+      </c>
+      <c r="CB1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_%DREB</t>
+        </is>
+      </c>
+      <c r="CC1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_%REB</t>
+        </is>
+      </c>
+      <c r="CD1" s="1" t="inlineStr">
+        <is>
+          <t>VISITANTE_PJ</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -592,88 +852,244 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.7932264412435124</v>
+        <v>0.79421905085401</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8992976359462221</v>
+        <v>0.8931077229714582</v>
       </c>
       <c r="E2" t="n">
-        <v>87.4664346378414</v>
+        <v>87.65138864477106</v>
       </c>
       <c r="F2" t="n">
-        <v>104.2302483697388</v>
+        <v>103.3387773577649</v>
       </c>
       <c r="G2" t="n">
-        <v>-16.7638137318974</v>
+        <v>-15.68738871299387</v>
       </c>
       <c r="H2" t="n">
-        <v>0.226156362485468</v>
+        <v>0.2287458374084601</v>
       </c>
       <c r="I2" t="n">
-        <v>0.6328018275900354</v>
+        <v>0.6365387046513382</v>
       </c>
       <c r="J2" t="n">
-        <v>0.4255063016022989</v>
+        <v>0.4284206934210179</v>
       </c>
       <c r="K2" t="n">
-        <v>4575</v>
+        <v>4775</v>
       </c>
       <c r="L2" t="n">
-        <v>1629</v>
+        <v>1703</v>
       </c>
       <c r="M2" t="n">
-        <v>422</v>
+        <v>445</v>
       </c>
       <c r="N2" t="n">
-        <v>916</v>
+        <v>958</v>
       </c>
       <c r="O2" t="n">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="P2" t="n">
-        <v>544</v>
+        <v>563</v>
       </c>
       <c r="Q2" t="n">
-        <v>341</v>
+        <v>354</v>
       </c>
       <c r="R2" t="n">
-        <v>520</v>
+        <v>542</v>
       </c>
       <c r="S2" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="T2" t="n">
-        <v>517</v>
+        <v>540</v>
       </c>
       <c r="U2" t="n">
-        <v>283</v>
+        <v>297</v>
       </c>
       <c r="V2" t="n">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="W2" t="n">
-        <v>372</v>
+        <v>392</v>
       </c>
       <c r="X2" t="n">
-        <v>525</v>
+        <v>551</v>
       </c>
       <c r="Y2" t="n">
-        <v>458</v>
+        <v>483</v>
       </c>
       <c r="Z2" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="AA2" t="n">
-        <v>1949</v>
+        <v>2020</v>
       </c>
       <c r="AB2" t="n">
-        <v>2060.8</v>
+        <v>2151.48</v>
       </c>
       <c r="AC2" t="n">
-        <v>1860.8</v>
+        <v>1941.48</v>
       </c>
       <c r="AD2" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>2275</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>227</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>469</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>72</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>261</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>175</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>275</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>93</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>252</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>129</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>89</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>167</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>267</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>237</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>11</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>1018</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>925</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>0.8325794091126206</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>0.9326252458599732</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>91.32082229766547</v>
+      </c>
+      <c r="AY2" t="n">
+        <v>108.5220535040225</v>
+      </c>
+      <c r="AZ2" t="n">
+        <v>-17.201231206357</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>0.2103867681662326</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>0.6233329813250507</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>0.4142152404063349</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>11</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>2500</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>218</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>489</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>81</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>302</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>179</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>267</v>
+      </c>
+      <c r="BL2" t="n">
+        <v>117</v>
+      </c>
+      <c r="BM2" t="n">
+        <v>288</v>
+      </c>
+      <c r="BN2" t="n">
+        <v>168</v>
+      </c>
+      <c r="BO2" t="n">
+        <v>109</v>
+      </c>
+      <c r="BP2" t="n">
+        <v>225</v>
+      </c>
+      <c r="BQ2" t="n">
+        <v>284</v>
+      </c>
+      <c r="BR2" t="n">
+        <v>246</v>
+      </c>
+      <c r="BS2" t="n">
+        <v>17</v>
+      </c>
+      <c r="BT2" t="n">
+        <v>1133.48</v>
+      </c>
+      <c r="BU2" t="n">
+        <v>1016.48</v>
+      </c>
+      <c r="BV2" t="n">
+        <v>0.7590553891169501</v>
+      </c>
+      <c r="BW2" t="n">
+        <v>0.8568833269903194</v>
+      </c>
+      <c r="BX2" t="n">
+        <v>84.28774112961786</v>
+      </c>
+      <c r="BY2" t="n">
+        <v>98.5874408903622</v>
+      </c>
+      <c r="BZ2" t="n">
+        <v>-14.29969976074433</v>
+      </c>
+      <c r="CA2" t="n">
+        <v>0.2455749842138355</v>
+      </c>
+      <c r="CB2" t="n">
+        <v>0.6486439510337686</v>
+      </c>
+      <c r="CC2" t="n">
+        <v>0.4414423586844773</v>
+      </c>
+      <c r="CD2" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="3">
@@ -688,88 +1104,244 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.7798389713717182</v>
+        <v>0.7788429133784546</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8769533715354867</v>
+        <v>0.8743056798289419</v>
       </c>
       <c r="E3" t="n">
-        <v>88.60003873601418</v>
+        <v>88.38814205594136</v>
       </c>
       <c r="F3" t="n">
-        <v>100.2015447008609</v>
+        <v>99.83279827026803</v>
       </c>
       <c r="G3" t="n">
-        <v>-11.60150596484677</v>
+        <v>-11.44465621432664</v>
       </c>
       <c r="H3" t="n">
-        <v>0.2825978129770437</v>
+        <v>0.2825392124128244</v>
       </c>
       <c r="I3" t="n">
-        <v>0.693671706083327</v>
+        <v>0.6945679673095176</v>
       </c>
       <c r="J3" t="n">
-        <v>0.4869005962403929</v>
+        <v>0.4877946001676438</v>
       </c>
       <c r="K3" t="n">
-        <v>4500</v>
+        <v>4700</v>
       </c>
       <c r="L3" t="n">
-        <v>1621</v>
+        <v>1692</v>
       </c>
       <c r="M3" t="n">
-        <v>437</v>
+        <v>452</v>
       </c>
       <c r="N3" t="n">
-        <v>949</v>
+        <v>989</v>
       </c>
       <c r="O3" t="n">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="P3" t="n">
-        <v>501</v>
+        <v>526</v>
       </c>
       <c r="Q3" t="n">
-        <v>369</v>
+        <v>386</v>
       </c>
       <c r="R3" t="n">
-        <v>587</v>
+        <v>607</v>
       </c>
       <c r="S3" t="n">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="T3" t="n">
-        <v>607</v>
+        <v>632</v>
       </c>
       <c r="U3" t="n">
-        <v>259</v>
+        <v>273</v>
       </c>
       <c r="V3" t="n">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="W3" t="n">
-        <v>366</v>
+        <v>386</v>
       </c>
       <c r="X3" t="n">
-        <v>511</v>
+        <v>536</v>
       </c>
       <c r="Y3" t="n">
-        <v>500</v>
+        <v>526</v>
       </c>
       <c r="Z3" t="n">
         <v>38</v>
       </c>
       <c r="AA3" t="n">
-        <v>1854</v>
+        <v>1928</v>
       </c>
       <c r="AB3" t="n">
-        <v>2074.28</v>
+        <v>2168.08</v>
       </c>
       <c r="AC3" t="n">
-        <v>1825.28</v>
+        <v>1910.08</v>
       </c>
       <c r="AD3" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>2425</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>225</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>520</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>64</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>278</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>191</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>291</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>141</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>298</v>
+      </c>
+      <c r="AN3" t="n">
+        <v>119</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>88</v>
+      </c>
+      <c r="AP3" t="n">
+        <v>195</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>269</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>262</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>18</v>
+      </c>
+      <c r="AT3" t="n">
+        <v>1121.04</v>
+      </c>
+      <c r="AU3" t="n">
+        <v>980.04</v>
+      </c>
+      <c r="AV3" t="n">
+        <v>0.7447167418509636</v>
+      </c>
+      <c r="AW3" t="n">
+        <v>0.9173596606819795</v>
+      </c>
+      <c r="AX3" t="n">
+        <v>85.18072152433017</v>
+      </c>
+      <c r="AY3" t="n">
+        <v>105.3200257751431</v>
+      </c>
+      <c r="AZ3" t="n">
+        <v>-20.1393042508129</v>
+      </c>
+      <c r="BA3" t="n">
+        <v>0.2893831029863625</v>
+      </c>
+      <c r="BB3" t="n">
+        <v>0.664883229227427</v>
+      </c>
+      <c r="BC3" t="n">
+        <v>0.4699609216836479</v>
+      </c>
+      <c r="BD3" t="n">
+        <v>12</v>
+      </c>
+      <c r="BE3" t="n">
+        <v>2275</v>
+      </c>
+      <c r="BF3" t="n">
+        <v>227</v>
+      </c>
+      <c r="BG3" t="n">
+        <v>469</v>
+      </c>
+      <c r="BH3" t="n">
+        <v>70</v>
+      </c>
+      <c r="BI3" t="n">
+        <v>248</v>
+      </c>
+      <c r="BJ3" t="n">
+        <v>195</v>
+      </c>
+      <c r="BK3" t="n">
+        <v>316</v>
+      </c>
+      <c r="BL3" t="n">
+        <v>117</v>
+      </c>
+      <c r="BM3" t="n">
+        <v>334</v>
+      </c>
+      <c r="BN3" t="n">
+        <v>154</v>
+      </c>
+      <c r="BO3" t="n">
+        <v>81</v>
+      </c>
+      <c r="BP3" t="n">
+        <v>191</v>
+      </c>
+      <c r="BQ3" t="n">
+        <v>267</v>
+      </c>
+      <c r="BR3" t="n">
+        <v>264</v>
+      </c>
+      <c r="BS3" t="n">
+        <v>20</v>
+      </c>
+      <c r="BT3" t="n">
+        <v>1047.04</v>
+      </c>
+      <c r="BU3" t="n">
+        <v>930.0400000000001</v>
+      </c>
+      <c r="BV3" t="n">
+        <v>0.8160714641357174</v>
+      </c>
+      <c r="BW3" t="n">
+        <v>0.8273377007165371</v>
+      </c>
+      <c r="BX3" t="n">
+        <v>91.88714627224449</v>
+      </c>
+      <c r="BY3" t="n">
+        <v>93.84673190131342</v>
+      </c>
+      <c r="BZ3" t="n">
+        <v>-1.959585629068915</v>
+      </c>
+      <c r="CA3" t="n">
+        <v>0.2750731499689644</v>
+      </c>
+      <c r="CB3" t="n">
+        <v>0.7269513179445258</v>
+      </c>
+      <c r="CC3" t="n">
+        <v>0.5072495221501847</v>
+      </c>
+      <c r="CD3" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -784,88 +1356,244 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.8609141374644953</v>
+        <v>0.8552340941452962</v>
       </c>
       <c r="D4" t="n">
-        <v>0.8569956194411837</v>
+        <v>0.8565393372336615</v>
       </c>
       <c r="E4" t="n">
-        <v>96.43103268080809</v>
+        <v>96.45266167279361</v>
       </c>
       <c r="F4" t="n">
-        <v>96.32674195563141</v>
+        <v>96.18436661761011</v>
       </c>
       <c r="G4" t="n">
-        <v>0.104290725176662</v>
+        <v>0.2682950551834975</v>
       </c>
       <c r="H4" t="n">
-        <v>0.276842720735008</v>
+        <v>0.2861350388654794</v>
       </c>
       <c r="I4" t="n">
-        <v>0.7227071598186717</v>
+        <v>0.7238938050439468</v>
       </c>
       <c r="J4" t="n">
-        <v>0.5015828769638487</v>
+        <v>0.50535037336184</v>
       </c>
       <c r="K4" t="n">
-        <v>4400</v>
+        <v>4600</v>
       </c>
       <c r="L4" t="n">
-        <v>1689</v>
+        <v>1766</v>
       </c>
       <c r="M4" t="n">
-        <v>378</v>
+        <v>396</v>
       </c>
       <c r="N4" t="n">
-        <v>789</v>
+        <v>837</v>
       </c>
       <c r="O4" t="n">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="P4" t="n">
-        <v>579</v>
+        <v>611</v>
       </c>
       <c r="Q4" t="n">
-        <v>378</v>
+        <v>398</v>
       </c>
       <c r="R4" t="n">
-        <v>554</v>
+        <v>580</v>
       </c>
       <c r="S4" t="n">
-        <v>209</v>
+        <v>235</v>
       </c>
       <c r="T4" t="n">
-        <v>564</v>
+        <v>588</v>
       </c>
       <c r="U4" t="n">
-        <v>307</v>
+        <v>320</v>
       </c>
       <c r="V4" t="n">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="W4" t="n">
-        <v>348</v>
+        <v>362</v>
       </c>
       <c r="X4" t="n">
-        <v>548</v>
+        <v>573</v>
       </c>
       <c r="Y4" t="n">
-        <v>502</v>
+        <v>529</v>
       </c>
       <c r="Z4" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="AA4" t="n">
-        <v>1677</v>
+        <v>1752</v>
       </c>
       <c r="AB4" t="n">
-        <v>1959.76</v>
+        <v>2065.2</v>
       </c>
       <c r="AC4" t="n">
-        <v>1750.76</v>
+        <v>1830.2</v>
       </c>
       <c r="AD4" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>2200</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>194</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>404</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>77</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>288</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>170</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>265</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>97</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>275</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>140</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>90</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>165</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>276</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>250</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>15</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>973.6</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>876.6</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>0.8112845099956398</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>0.8427723790680651</v>
+      </c>
+      <c r="AX4" t="n">
+        <v>90.0643309952619</v>
+      </c>
+      <c r="AY4" t="n">
+        <v>94.94027726900917</v>
+      </c>
+      <c r="AZ4" t="n">
+        <v>-4.875946273747268</v>
+      </c>
+      <c r="BA4" t="n">
+        <v>0.2579706936183871</v>
+      </c>
+      <c r="BB4" t="n">
+        <v>0.7094003932538758</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>0.4840333923164064</v>
+      </c>
+      <c r="BD4" t="n">
+        <v>11</v>
+      </c>
+      <c r="BE4" t="n">
+        <v>2400</v>
+      </c>
+      <c r="BF4" t="n">
+        <v>202</v>
+      </c>
+      <c r="BG4" t="n">
+        <v>433</v>
+      </c>
+      <c r="BH4" t="n">
+        <v>115</v>
+      </c>
+      <c r="BI4" t="n">
+        <v>323</v>
+      </c>
+      <c r="BJ4" t="n">
+        <v>228</v>
+      </c>
+      <c r="BK4" t="n">
+        <v>315</v>
+      </c>
+      <c r="BL4" t="n">
+        <v>138</v>
+      </c>
+      <c r="BM4" t="n">
+        <v>313</v>
+      </c>
+      <c r="BN4" t="n">
+        <v>180</v>
+      </c>
+      <c r="BO4" t="n">
+        <v>93</v>
+      </c>
+      <c r="BP4" t="n">
+        <v>197</v>
+      </c>
+      <c r="BQ4" t="n">
+        <v>297</v>
+      </c>
+      <c r="BR4" t="n">
+        <v>279</v>
+      </c>
+      <c r="BS4" t="n">
+        <v>15</v>
+      </c>
+      <c r="BT4" t="n">
+        <v>1091.6</v>
+      </c>
+      <c r="BU4" t="n">
+        <v>953.6</v>
+      </c>
+      <c r="BV4" t="n">
+        <v>0.8955212129491478</v>
+      </c>
+      <c r="BW4" t="n">
+        <v>0.8691590488854583</v>
+      </c>
+      <c r="BX4" t="n">
+        <v>102.308631460531</v>
+      </c>
+      <c r="BY4" t="n">
+        <v>97.32478185382764</v>
+      </c>
+      <c r="BZ4" t="n">
+        <v>4.983849606703366</v>
+      </c>
+      <c r="CA4" t="n">
+        <v>0.3119523553419807</v>
+      </c>
+      <c r="CB4" t="n">
+        <v>0.7371794325181783</v>
+      </c>
+      <c r="CC4" t="n">
+        <v>0.5248909393201541</v>
+      </c>
+      <c r="CD4" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="5">
@@ -963,6 +1691,162 @@
       <c r="AD5" t="n">
         <v>22</v>
       </c>
+      <c r="AE5" t="n">
+        <v>2400</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>218</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>465</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>72</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>306</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>152</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>261</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>105</v>
+      </c>
+      <c r="AM5" t="n">
+        <v>318</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>150</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>108</v>
+      </c>
+      <c r="AP5" t="n">
+        <v>173</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>261</v>
+      </c>
+      <c r="AR5" t="n">
+        <v>231</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>23</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>1058.84</v>
+      </c>
+      <c r="AU5" t="n">
+        <v>953.84</v>
+      </c>
+      <c r="AV5" t="n">
+        <v>0.7609639197224817</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>0.8300582054482447</v>
+      </c>
+      <c r="AX5" t="n">
+        <v>84.47980423604744</v>
+      </c>
+      <c r="AY5" t="n">
+        <v>94.89754631805302</v>
+      </c>
+      <c r="AZ5" t="n">
+        <v>-10.4177420820056</v>
+      </c>
+      <c r="BA5" t="n">
+        <v>0.2248932579416265</v>
+      </c>
+      <c r="BB5" t="n">
+        <v>0.7055990021296555</v>
+      </c>
+      <c r="BC5" t="n">
+        <v>0.4646934272215936</v>
+      </c>
+      <c r="BD5" t="n">
+        <v>12</v>
+      </c>
+      <c r="BE5" t="n">
+        <v>2000</v>
+      </c>
+      <c r="BF5" t="n">
+        <v>195</v>
+      </c>
+      <c r="BG5" t="n">
+        <v>399</v>
+      </c>
+      <c r="BH5" t="n">
+        <v>72</v>
+      </c>
+      <c r="BI5" t="n">
+        <v>239</v>
+      </c>
+      <c r="BJ5" t="n">
+        <v>129</v>
+      </c>
+      <c r="BK5" t="n">
+        <v>200</v>
+      </c>
+      <c r="BL5" t="n">
+        <v>94</v>
+      </c>
+      <c r="BM5" t="n">
+        <v>250</v>
+      </c>
+      <c r="BN5" t="n">
+        <v>143</v>
+      </c>
+      <c r="BO5" t="n">
+        <v>78</v>
+      </c>
+      <c r="BP5" t="n">
+        <v>144</v>
+      </c>
+      <c r="BQ5" t="n">
+        <v>226</v>
+      </c>
+      <c r="BR5" t="n">
+        <v>189</v>
+      </c>
+      <c r="BS5" t="n">
+        <v>34</v>
+      </c>
+      <c r="BT5" t="n">
+        <v>870</v>
+      </c>
+      <c r="BU5" t="n">
+        <v>776</v>
+      </c>
+      <c r="BV5" t="n">
+        <v>0.8497493654267423</v>
+      </c>
+      <c r="BW5" t="n">
+        <v>0.8659530476704186</v>
+      </c>
+      <c r="BX5" t="n">
+        <v>95.18769127030717</v>
+      </c>
+      <c r="BY5" t="n">
+        <v>99.52050065476222</v>
+      </c>
+      <c r="BZ5" t="n">
+        <v>-4.332809384455037</v>
+      </c>
+      <c r="CA5" t="n">
+        <v>0.2753194409663689</v>
+      </c>
+      <c r="CB5" t="n">
+        <v>0.6797123057390178</v>
+      </c>
+      <c r="CC5" t="n">
+        <v>0.4824204316939832</v>
+      </c>
+      <c r="CD5" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1059,6 +1943,162 @@
       <c r="AD6" t="n">
         <v>22</v>
       </c>
+      <c r="AE6" t="n">
+        <v>2225</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>193</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>402</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>88</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>306</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>212</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>286</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>124</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>247</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>144</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>92</v>
+      </c>
+      <c r="AP6" t="n">
+        <v>161</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>240</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>251</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>32</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>994.84</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>870.84</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>0.86869424566162</v>
+      </c>
+      <c r="AW6" t="n">
+        <v>0.9001813857681568</v>
+      </c>
+      <c r="AX6" t="n">
+        <v>99.21282133313046</v>
+      </c>
+      <c r="AY6" t="n">
+        <v>103.2737218897539</v>
+      </c>
+      <c r="AZ6" t="n">
+        <v>-4.060900556623451</v>
+      </c>
+      <c r="BA6" t="n">
+        <v>0.3023873469761691</v>
+      </c>
+      <c r="BB6" t="n">
+        <v>0.6554273861291534</v>
+      </c>
+      <c r="BC6" t="n">
+        <v>0.4714508141145842</v>
+      </c>
+      <c r="BD6" t="n">
+        <v>11</v>
+      </c>
+      <c r="BE6" t="n">
+        <v>2200</v>
+      </c>
+      <c r="BF6" t="n">
+        <v>185</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>393</v>
+      </c>
+      <c r="BH6" t="n">
+        <v>98</v>
+      </c>
+      <c r="BI6" t="n">
+        <v>308</v>
+      </c>
+      <c r="BJ6" t="n">
+        <v>195</v>
+      </c>
+      <c r="BK6" t="n">
+        <v>274</v>
+      </c>
+      <c r="BL6" t="n">
+        <v>141</v>
+      </c>
+      <c r="BM6" t="n">
+        <v>288</v>
+      </c>
+      <c r="BN6" t="n">
+        <v>142</v>
+      </c>
+      <c r="BO6" t="n">
+        <v>102</v>
+      </c>
+      <c r="BP6" t="n">
+        <v>147</v>
+      </c>
+      <c r="BQ6" t="n">
+        <v>219</v>
+      </c>
+      <c r="BR6" t="n">
+        <v>248</v>
+      </c>
+      <c r="BS6" t="n">
+        <v>41</v>
+      </c>
+      <c r="BT6" t="n">
+        <v>968.5599999999999</v>
+      </c>
+      <c r="BU6" t="n">
+        <v>827.5599999999999</v>
+      </c>
+      <c r="BV6" t="n">
+        <v>0.8889125882110558</v>
+      </c>
+      <c r="BW6" t="n">
+        <v>0.8044988712324487</v>
+      </c>
+      <c r="BX6" t="n">
+        <v>103.6628342555971</v>
+      </c>
+      <c r="BY6" t="n">
+        <v>90.65068987236315</v>
+      </c>
+      <c r="BZ6" t="n">
+        <v>13.01214438323399</v>
+      </c>
+      <c r="CA6" t="n">
+        <v>0.3404160576951831</v>
+      </c>
+      <c r="CB6" t="n">
+        <v>0.7251482951140941</v>
+      </c>
+      <c r="CC6" t="n">
+        <v>0.5324210545722137</v>
+      </c>
+      <c r="CD6" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1155,6 +2195,162 @@
       <c r="AD7" t="n">
         <v>22</v>
       </c>
+      <c r="AE7" t="n">
+        <v>2225</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>203</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>423</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>105</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>311</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>189</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>307</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>149</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>266</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>162</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>107</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>135</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>266</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>257</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>29</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>1004.08</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>855.08</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>0.9090901349216334</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>0.7725100510678167</v>
+      </c>
+      <c r="AX7" t="n">
+        <v>106.5743399536909</v>
+      </c>
+      <c r="AY7" t="n">
+        <v>90.05926312319251</v>
+      </c>
+      <c r="AZ7" t="n">
+        <v>16.51507683049837</v>
+      </c>
+      <c r="BA7" t="n">
+        <v>0.3660971155739813</v>
+      </c>
+      <c r="BB7" t="n">
+        <v>0.6584750752269134</v>
+      </c>
+      <c r="BC7" t="n">
+        <v>0.5141991181747219</v>
+      </c>
+      <c r="BD7" t="n">
+        <v>11</v>
+      </c>
+      <c r="BE7" t="n">
+        <v>2225</v>
+      </c>
+      <c r="BF7" t="n">
+        <v>238</v>
+      </c>
+      <c r="BG7" t="n">
+        <v>457</v>
+      </c>
+      <c r="BH7" t="n">
+        <v>75</v>
+      </c>
+      <c r="BI7" t="n">
+        <v>291</v>
+      </c>
+      <c r="BJ7" t="n">
+        <v>171</v>
+      </c>
+      <c r="BK7" t="n">
+        <v>251</v>
+      </c>
+      <c r="BL7" t="n">
+        <v>139</v>
+      </c>
+      <c r="BM7" t="n">
+        <v>283</v>
+      </c>
+      <c r="BN7" t="n">
+        <v>170</v>
+      </c>
+      <c r="BO7" t="n">
+        <v>139</v>
+      </c>
+      <c r="BP7" t="n">
+        <v>145</v>
+      </c>
+      <c r="BQ7" t="n">
+        <v>251</v>
+      </c>
+      <c r="BR7" t="n">
+        <v>228</v>
+      </c>
+      <c r="BS7" t="n">
+        <v>36</v>
+      </c>
+      <c r="BT7" t="n">
+        <v>1003.44</v>
+      </c>
+      <c r="BU7" t="n">
+        <v>864.4399999999999</v>
+      </c>
+      <c r="BV7" t="n">
+        <v>0.8707625284534896</v>
+      </c>
+      <c r="BW7" t="n">
+        <v>0.7404079264289493</v>
+      </c>
+      <c r="BX7" t="n">
+        <v>100.873034714564</v>
+      </c>
+      <c r="BY7" t="n">
+        <v>83.00693417814875</v>
+      </c>
+      <c r="BZ7" t="n">
+        <v>17.86610053641522</v>
+      </c>
+      <c r="CA7" t="n">
+        <v>0.3416891558818338</v>
+      </c>
+      <c r="CB7" t="n">
+        <v>0.729813023126999</v>
+      </c>
+      <c r="CC7" t="n">
+        <v>0.5301654327429968</v>
+      </c>
+      <c r="CD7" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1251,6 +2447,162 @@
       <c r="AD8" t="n">
         <v>22</v>
       </c>
+      <c r="AE8" t="n">
+        <v>2200</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>225</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>430</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>107</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>316</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>164</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>275</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>124</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>236</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>172</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>111</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>142</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>249</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>252</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>34</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>1009</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>885</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>0.9253628591597004</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>0.9093653200407121</v>
+      </c>
+      <c r="AX8" t="n">
+        <v>105.4136550526525</v>
+      </c>
+      <c r="AY8" t="n">
+        <v>102.410289398452</v>
+      </c>
+      <c r="AZ8" t="n">
+        <v>3.003365654200495</v>
+      </c>
+      <c r="BA8" t="n">
+        <v>0.3089596745490724</v>
+      </c>
+      <c r="BB8" t="n">
+        <v>0.6811995161557435</v>
+      </c>
+      <c r="BC8" t="n">
+        <v>0.4853324056179123</v>
+      </c>
+      <c r="BD8" t="n">
+        <v>11</v>
+      </c>
+      <c r="BE8" t="n">
+        <v>2200</v>
+      </c>
+      <c r="BF8" t="n">
+        <v>251</v>
+      </c>
+      <c r="BG8" t="n">
+        <v>439</v>
+      </c>
+      <c r="BH8" t="n">
+        <v>114</v>
+      </c>
+      <c r="BI8" t="n">
+        <v>315</v>
+      </c>
+      <c r="BJ8" t="n">
+        <v>177</v>
+      </c>
+      <c r="BK8" t="n">
+        <v>259</v>
+      </c>
+      <c r="BL8" t="n">
+        <v>135</v>
+      </c>
+      <c r="BM8" t="n">
+        <v>311</v>
+      </c>
+      <c r="BN8" t="n">
+        <v>174</v>
+      </c>
+      <c r="BO8" t="n">
+        <v>101</v>
+      </c>
+      <c r="BP8" t="n">
+        <v>176</v>
+      </c>
+      <c r="BQ8" t="n">
+        <v>252</v>
+      </c>
+      <c r="BR8" t="n">
+        <v>229</v>
+      </c>
+      <c r="BS8" t="n">
+        <v>25</v>
+      </c>
+      <c r="BT8" t="n">
+        <v>1043.96</v>
+      </c>
+      <c r="BU8" t="n">
+        <v>908.96</v>
+      </c>
+      <c r="BV8" t="n">
+        <v>0.9768864975052385</v>
+      </c>
+      <c r="BW8" t="n">
+        <v>0.8381641429136938</v>
+      </c>
+      <c r="BX8" t="n">
+        <v>112.4975467875901</v>
+      </c>
+      <c r="BY8" t="n">
+        <v>94.55467491312605</v>
+      </c>
+      <c r="BZ8" t="n">
+        <v>17.94287187446406</v>
+      </c>
+      <c r="CA8" t="n">
+        <v>0.3628221481796532</v>
+      </c>
+      <c r="CB8" t="n">
+        <v>0.7329371046994038</v>
+      </c>
+      <c r="CC8" t="n">
+        <v>0.558600385217771</v>
+      </c>
+      <c r="CD8" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1347,6 +2699,162 @@
       <c r="AD9" t="n">
         <v>22</v>
       </c>
+      <c r="AE9" t="n">
+        <v>2250</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>224</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>463</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>88</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>287</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>185</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>260</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>122</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>246</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>128</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>75</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>154</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>282</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>234</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>16</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>1018.4</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>896.4</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>0.8924302470204059</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>0.916204087882969</v>
+      </c>
+      <c r="AX9" t="n">
+        <v>100.681634986238</v>
+      </c>
+      <c r="AY9" t="n">
+        <v>103.8540478338802</v>
+      </c>
+      <c r="AZ9" t="n">
+        <v>-3.172412847642221</v>
+      </c>
+      <c r="BA9" t="n">
+        <v>0.2805952855821541</v>
+      </c>
+      <c r="BB9" t="n">
+        <v>0.6683499037971179</v>
+      </c>
+      <c r="BC9" t="n">
+        <v>0.4608105522848097</v>
+      </c>
+      <c r="BD9" t="n">
+        <v>11</v>
+      </c>
+      <c r="BE9" t="n">
+        <v>2225</v>
+      </c>
+      <c r="BF9" t="n">
+        <v>209</v>
+      </c>
+      <c r="BG9" t="n">
+        <v>419</v>
+      </c>
+      <c r="BH9" t="n">
+        <v>98</v>
+      </c>
+      <c r="BI9" t="n">
+        <v>309</v>
+      </c>
+      <c r="BJ9" t="n">
+        <v>185</v>
+      </c>
+      <c r="BK9" t="n">
+        <v>261</v>
+      </c>
+      <c r="BL9" t="n">
+        <v>120</v>
+      </c>
+      <c r="BM9" t="n">
+        <v>288</v>
+      </c>
+      <c r="BN9" t="n">
+        <v>125</v>
+      </c>
+      <c r="BO9" t="n">
+        <v>98</v>
+      </c>
+      <c r="BP9" t="n">
+        <v>176</v>
+      </c>
+      <c r="BQ9" t="n">
+        <v>281</v>
+      </c>
+      <c r="BR9" t="n">
+        <v>247</v>
+      </c>
+      <c r="BS9" t="n">
+        <v>21</v>
+      </c>
+      <c r="BT9" t="n">
+        <v>1018.84</v>
+      </c>
+      <c r="BU9" t="n">
+        <v>898.8399999999999</v>
+      </c>
+      <c r="BV9" t="n">
+        <v>0.8847417279158093</v>
+      </c>
+      <c r="BW9" t="n">
+        <v>0.8726908458129556</v>
+      </c>
+      <c r="BX9" t="n">
+        <v>100.0965245505916</v>
+      </c>
+      <c r="BY9" t="n">
+        <v>100.8269359778485</v>
+      </c>
+      <c r="BZ9" t="n">
+        <v>-0.7304114272569897</v>
+      </c>
+      <c r="CA9" t="n">
+        <v>0.3019295435579464</v>
+      </c>
+      <c r="CB9" t="n">
+        <v>0.6788325578583657</v>
+      </c>
+      <c r="CC9" t="n">
+        <v>0.496100939586104</v>
+      </c>
+      <c r="CD9" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1360,88 +2868,244 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.8133013749223772</v>
+        <v>0.8157211956343801</v>
       </c>
       <c r="D10" t="n">
-        <v>0.871750130415911</v>
+        <v>0.8671414328768302</v>
       </c>
       <c r="E10" t="n">
-        <v>92.15516956181369</v>
+        <v>92.25459836921318</v>
       </c>
       <c r="F10" t="n">
-        <v>97.11729209044762</v>
+        <v>96.88363240243056</v>
       </c>
       <c r="G10" t="n">
-        <v>-4.962122528633909</v>
+        <v>-4.629034033217362</v>
       </c>
       <c r="H10" t="n">
-        <v>0.2915979078853461</v>
+        <v>0.2883204430301665</v>
       </c>
       <c r="I10" t="n">
-        <v>0.7362647496035581</v>
+        <v>0.7270793257077512</v>
       </c>
       <c r="J10" t="n">
-        <v>0.5042018536195352</v>
+        <v>0.4986549633153544</v>
       </c>
       <c r="K10" t="n">
-        <v>4475</v>
+        <v>4675</v>
       </c>
       <c r="L10" t="n">
-        <v>1640</v>
+        <v>1727</v>
       </c>
       <c r="M10" t="n">
-        <v>404</v>
+        <v>429</v>
       </c>
       <c r="N10" t="n">
-        <v>862</v>
+        <v>910</v>
       </c>
       <c r="O10" t="n">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="P10" t="n">
-        <v>570</v>
+        <v>592</v>
       </c>
       <c r="Q10" t="n">
-        <v>340</v>
+        <v>359</v>
       </c>
       <c r="R10" t="n">
-        <v>526</v>
+        <v>549</v>
       </c>
       <c r="S10" t="n">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="T10" t="n">
-        <v>552</v>
+        <v>573</v>
       </c>
       <c r="U10" t="n">
-        <v>332</v>
+        <v>350</v>
       </c>
       <c r="V10" t="n">
-        <v>229</v>
+        <v>250</v>
       </c>
       <c r="W10" t="n">
-        <v>363</v>
+        <v>383</v>
       </c>
       <c r="X10" t="n">
-        <v>496</v>
+        <v>514</v>
       </c>
       <c r="Y10" t="n">
+        <v>504</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>34</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>1804</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>2126.56</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>1876.56</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>23</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>2450</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>214</v>
+      </c>
+      <c r="AG10" t="n">
         <v>486</v>
       </c>
-      <c r="Z10" t="n">
-        <v>33</v>
-      </c>
-      <c r="AA10" t="n">
-        <v>1716</v>
-      </c>
-      <c r="AB10" t="n">
-        <v>2026.44</v>
-      </c>
-      <c r="AC10" t="n">
-        <v>1784.44</v>
-      </c>
-      <c r="AD10" t="n">
-        <v>22</v>
+      <c r="AH10" t="n">
+        <v>88</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>299</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>194</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>298</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>142</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>308</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>185</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>128</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>213</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>262</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>265</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>16</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>1129.12</v>
+      </c>
+      <c r="AU10" t="n">
+        <v>987.12</v>
+      </c>
+      <c r="AV10" t="n">
+        <v>0.7874884738876604</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>0.8640924156729811</v>
+      </c>
+      <c r="AX10" t="n">
+        <v>89.845713417261</v>
+      </c>
+      <c r="AY10" t="n">
+        <v>96.15271479759168</v>
+      </c>
+      <c r="AZ10" t="n">
+        <v>-6.307001380330674</v>
+      </c>
+      <c r="BA10" t="n">
+        <v>0.2993406720134754</v>
+      </c>
+      <c r="BB10" t="n">
+        <v>0.7458962851115857</v>
+      </c>
+      <c r="BC10" t="n">
+        <v>0.5081427539148284</v>
+      </c>
+      <c r="BD10" t="n">
+        <v>12</v>
+      </c>
+      <c r="BE10" t="n">
+        <v>2225</v>
+      </c>
+      <c r="BF10" t="n">
+        <v>215</v>
+      </c>
+      <c r="BG10" t="n">
+        <v>424</v>
+      </c>
+      <c r="BH10" t="n">
+        <v>82</v>
+      </c>
+      <c r="BI10" t="n">
+        <v>293</v>
+      </c>
+      <c r="BJ10" t="n">
+        <v>165</v>
+      </c>
+      <c r="BK10" t="n">
+        <v>251</v>
+      </c>
+      <c r="BL10" t="n">
+        <v>108</v>
+      </c>
+      <c r="BM10" t="n">
+        <v>265</v>
+      </c>
+      <c r="BN10" t="n">
+        <v>165</v>
+      </c>
+      <c r="BO10" t="n">
+        <v>122</v>
+      </c>
+      <c r="BP10" t="n">
+        <v>170</v>
+      </c>
+      <c r="BQ10" t="n">
+        <v>252</v>
+      </c>
+      <c r="BR10" t="n">
+        <v>239</v>
+      </c>
+      <c r="BS10" t="n">
+        <v>18</v>
+      </c>
+      <c r="BT10" t="n">
+        <v>997.4400000000001</v>
+      </c>
+      <c r="BU10" t="n">
+        <v>889.4400000000001</v>
+      </c>
+      <c r="BV10" t="n">
+        <v>0.8465205284489834</v>
+      </c>
+      <c r="BW10" t="n">
+        <v>0.8704676334628471</v>
+      </c>
+      <c r="BX10" t="n">
+        <v>94.88247286225192</v>
+      </c>
+      <c r="BY10" t="n">
+        <v>97.68099706225476</v>
+      </c>
+      <c r="BZ10" t="n">
+        <v>-2.79852420000284</v>
+      </c>
+      <c r="CA10" t="n">
+        <v>0.276298375048375</v>
+      </c>
+      <c r="CB10" t="n">
+        <v>0.7065517336308411</v>
+      </c>
+      <c r="CC10" t="n">
+        <v>0.4883046462977463</v>
+      </c>
+      <c r="CD10" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="11">
@@ -1456,88 +3120,244 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.8659964842198242</v>
+        <v>0.8651488600654045</v>
       </c>
       <c r="D11" t="n">
-        <v>0.8894924049662237</v>
+        <v>0.8825698282773843</v>
       </c>
       <c r="E11" t="n">
-        <v>99.16802165723639</v>
+        <v>98.90211241914531</v>
       </c>
       <c r="F11" t="n">
-        <v>99.22541318456575</v>
+        <v>99.12554737204009</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.05739152732933597</v>
+        <v>-0.2234349528947509</v>
       </c>
       <c r="H11" t="n">
-        <v>0.3182660895611033</v>
+        <v>0.3152979987106205</v>
       </c>
       <c r="I11" t="n">
-        <v>0.7324637522385526</v>
+        <v>0.7227668048483613</v>
       </c>
       <c r="J11" t="n">
-        <v>0.5223887144796326</v>
+        <v>0.5175789749754031</v>
       </c>
       <c r="K11" t="n">
-        <v>4425</v>
+        <v>4625</v>
       </c>
       <c r="L11" t="n">
-        <v>1715</v>
+        <v>1790</v>
       </c>
       <c r="M11" t="n">
-        <v>421</v>
+        <v>438</v>
       </c>
       <c r="N11" t="n">
-        <v>862</v>
+        <v>898</v>
       </c>
       <c r="O11" t="n">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="P11" t="n">
-        <v>554</v>
+        <v>573</v>
       </c>
       <c r="Q11" t="n">
-        <v>336</v>
+        <v>365</v>
       </c>
       <c r="R11" t="n">
-        <v>517</v>
+        <v>557</v>
       </c>
       <c r="S11" t="n">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="T11" t="n">
-        <v>541</v>
+        <v>568</v>
       </c>
       <c r="U11" t="n">
-        <v>301</v>
+        <v>312</v>
       </c>
       <c r="V11" t="n">
-        <v>184</v>
+        <v>194</v>
       </c>
       <c r="W11" t="n">
-        <v>330</v>
+        <v>346</v>
       </c>
       <c r="X11" t="n">
-        <v>502</v>
+        <v>529</v>
       </c>
       <c r="Y11" t="n">
-        <v>473</v>
+        <v>498</v>
       </c>
       <c r="Z11" t="n">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="AA11" t="n">
-        <v>1717</v>
+        <v>1794</v>
       </c>
       <c r="AB11" t="n">
-        <v>1973.48</v>
+        <v>2062.08</v>
       </c>
       <c r="AC11" t="n">
-        <v>1726.48</v>
+        <v>1807.08</v>
       </c>
       <c r="AD11" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>2200</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>208</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>423</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>81</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>262</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>182</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>265</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>112</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>278</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>144</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>91</v>
+      </c>
+      <c r="AP11" t="n">
+        <v>178</v>
+      </c>
+      <c r="AQ11" t="n">
+        <v>250</v>
+      </c>
+      <c r="AR11" t="n">
+        <v>236</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>23</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>979.6</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>867.6</v>
+      </c>
+      <c r="AV11" t="n">
+        <v>0.8548206842280048</v>
+      </c>
+      <c r="AW11" t="n">
+        <v>0.8645562443169893</v>
+      </c>
+      <c r="AX11" t="n">
+        <v>96.5053428133982</v>
+      </c>
+      <c r="AY11" t="n">
+        <v>99.03797808924797</v>
+      </c>
+      <c r="AZ11" t="n">
+        <v>-2.532635275849762</v>
+      </c>
+      <c r="BA11" t="n">
+        <v>0.2890379628790085</v>
+      </c>
+      <c r="BB11" t="n">
+        <v>0.6919336187785066</v>
+      </c>
+      <c r="BC11" t="n">
+        <v>0.4959883724417103</v>
+      </c>
+      <c r="BD11" t="n">
+        <v>11</v>
+      </c>
+      <c r="BE11" t="n">
+        <v>2425</v>
+      </c>
+      <c r="BF11" t="n">
+        <v>230</v>
+      </c>
+      <c r="BG11" t="n">
+        <v>475</v>
+      </c>
+      <c r="BH11" t="n">
+        <v>102</v>
+      </c>
+      <c r="BI11" t="n">
+        <v>311</v>
+      </c>
+      <c r="BJ11" t="n">
+        <v>183</v>
+      </c>
+      <c r="BK11" t="n">
+        <v>292</v>
+      </c>
+      <c r="BL11" t="n">
+        <v>143</v>
+      </c>
+      <c r="BM11" t="n">
+        <v>290</v>
+      </c>
+      <c r="BN11" t="n">
+        <v>168</v>
+      </c>
+      <c r="BO11" t="n">
+        <v>103</v>
+      </c>
+      <c r="BP11" t="n">
+        <v>168</v>
+      </c>
+      <c r="BQ11" t="n">
+        <v>279</v>
+      </c>
+      <c r="BR11" t="n">
+        <v>262</v>
+      </c>
+      <c r="BS11" t="n">
+        <v>26</v>
+      </c>
+      <c r="BT11" t="n">
+        <v>1082.48</v>
+      </c>
+      <c r="BU11" t="n">
+        <v>939.48</v>
+      </c>
+      <c r="BV11" t="n">
+        <v>0.8746163545830208</v>
+      </c>
+      <c r="BW11" t="n">
+        <v>0.8990822802410793</v>
+      </c>
+      <c r="BX11" t="n">
+        <v>101.0991512244135</v>
+      </c>
+      <c r="BY11" t="n">
+        <v>99.20581921459949</v>
+      </c>
+      <c r="BZ11" t="n">
+        <v>1.893332009814009</v>
+      </c>
+      <c r="CA11" t="n">
+        <v>0.3393696982229317</v>
+      </c>
+      <c r="CB11" t="n">
+        <v>0.7510305587457284</v>
+      </c>
+      <c r="CC11" t="n">
+        <v>0.537370360631288</v>
+      </c>
+      <c r="CD11" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="12">
@@ -1635,6 +3455,162 @@
       <c r="AD12" t="n">
         <v>22</v>
       </c>
+      <c r="AE12" t="n">
+        <v>2225</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>189</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>409</v>
+      </c>
+      <c r="AH12" t="n">
+        <v>78</v>
+      </c>
+      <c r="AI12" t="n">
+        <v>276</v>
+      </c>
+      <c r="AJ12" t="n">
+        <v>207</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>332</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>117</v>
+      </c>
+      <c r="AM12" t="n">
+        <v>297</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>168</v>
+      </c>
+      <c r="AO12" t="n">
+        <v>94</v>
+      </c>
+      <c r="AP12" t="n">
+        <v>161</v>
+      </c>
+      <c r="AQ12" t="n">
+        <v>214</v>
+      </c>
+      <c r="AR12" t="n">
+        <v>264</v>
+      </c>
+      <c r="AS12" t="n">
+        <v>16</v>
+      </c>
+      <c r="AT12" t="n">
+        <v>992.08</v>
+      </c>
+      <c r="AU12" t="n">
+        <v>875.08</v>
+      </c>
+      <c r="AV12" t="n">
+        <v>0.8326150419113723</v>
+      </c>
+      <c r="AW12" t="n">
+        <v>0.8132670660103916</v>
+      </c>
+      <c r="AX12" t="n">
+        <v>93.75148197408929</v>
+      </c>
+      <c r="AY12" t="n">
+        <v>94.77946658778515</v>
+      </c>
+      <c r="AZ12" t="n">
+        <v>-1.027984613695842</v>
+      </c>
+      <c r="BA12" t="n">
+        <v>0.2698945497370477</v>
+      </c>
+      <c r="BB12" t="n">
+        <v>0.6739685297548448</v>
+      </c>
+      <c r="BC12" t="n">
+        <v>0.4802046638684241</v>
+      </c>
+      <c r="BD12" t="n">
+        <v>11</v>
+      </c>
+      <c r="BE12" t="n">
+        <v>2225</v>
+      </c>
+      <c r="BF12" t="n">
+        <v>205</v>
+      </c>
+      <c r="BG12" t="n">
+        <v>405</v>
+      </c>
+      <c r="BH12" t="n">
+        <v>87</v>
+      </c>
+      <c r="BI12" t="n">
+        <v>290</v>
+      </c>
+      <c r="BJ12" t="n">
+        <v>179</v>
+      </c>
+      <c r="BK12" t="n">
+        <v>274</v>
+      </c>
+      <c r="BL12" t="n">
+        <v>114</v>
+      </c>
+      <c r="BM12" t="n">
+        <v>300</v>
+      </c>
+      <c r="BN12" t="n">
+        <v>181</v>
+      </c>
+      <c r="BO12" t="n">
+        <v>89</v>
+      </c>
+      <c r="BP12" t="n">
+        <v>181</v>
+      </c>
+      <c r="BQ12" t="n">
+        <v>232</v>
+      </c>
+      <c r="BR12" t="n">
+        <v>230</v>
+      </c>
+      <c r="BS12" t="n">
+        <v>20</v>
+      </c>
+      <c r="BT12" t="n">
+        <v>996.5599999999999</v>
+      </c>
+      <c r="BU12" t="n">
+        <v>882.5599999999999</v>
+      </c>
+      <c r="BV12" t="n">
+        <v>0.8545907026542751</v>
+      </c>
+      <c r="BW12" t="n">
+        <v>0.8295703444047248</v>
+      </c>
+      <c r="BX12" t="n">
+        <v>96.45771050675101</v>
+      </c>
+      <c r="BY12" t="n">
+        <v>95.65050799610221</v>
+      </c>
+      <c r="BZ12" t="n">
+        <v>0.8072025106488018</v>
+      </c>
+      <c r="CA12" t="n">
+        <v>0.2964350580724492</v>
+      </c>
+      <c r="CB12" t="n">
+        <v>0.6832061096070086</v>
+      </c>
+      <c r="CC12" t="n">
+        <v>0.5047904799075101</v>
+      </c>
+      <c r="CD12" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1648,88 +3624,244 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.764152160435032</v>
+        <v>0.7618110407067801</v>
       </c>
       <c r="D13" t="n">
-        <v>0.8320716013647623</v>
+        <v>0.8365592782562316</v>
       </c>
       <c r="E13" t="n">
-        <v>86.83287074287749</v>
+        <v>86.42742413597821</v>
       </c>
       <c r="F13" t="n">
-        <v>94.78885824270829</v>
+        <v>95.2560109870852</v>
       </c>
       <c r="G13" t="n">
-        <v>-7.955987499830806</v>
+        <v>-8.828586851106968</v>
       </c>
       <c r="H13" t="n">
-        <v>0.3015342644310964</v>
+        <v>0.2963292173609696</v>
       </c>
       <c r="I13" t="n">
-        <v>0.7173783052805086</v>
+        <v>0.7196327602348679</v>
       </c>
       <c r="J13" t="n">
-        <v>0.520495594230318</v>
+        <v>0.5196044814376954</v>
       </c>
       <c r="K13" t="n">
-        <v>4425</v>
+        <v>4625</v>
       </c>
       <c r="L13" t="n">
-        <v>1533</v>
+        <v>1584</v>
       </c>
       <c r="M13" t="n">
-        <v>408</v>
+        <v>418</v>
       </c>
       <c r="N13" t="n">
-        <v>901</v>
+        <v>927</v>
       </c>
       <c r="O13" t="n">
+        <v>137</v>
+      </c>
+      <c r="P13" t="n">
+        <v>491</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>337</v>
+      </c>
+      <c r="R13" t="n">
+        <v>583</v>
+      </c>
+      <c r="S13" t="n">
+        <v>247</v>
+      </c>
+      <c r="T13" t="n">
+        <v>669</v>
+      </c>
+      <c r="U13" t="n">
+        <v>261</v>
+      </c>
+      <c r="V13" t="n">
         <v>131</v>
       </c>
-      <c r="P13" t="n">
-        <v>465</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>324</v>
-      </c>
-      <c r="R13" t="n">
-        <v>563</v>
-      </c>
-      <c r="S13" t="n">
-        <v>241</v>
-      </c>
-      <c r="T13" t="n">
-        <v>639</v>
-      </c>
-      <c r="U13" t="n">
-        <v>255</v>
-      </c>
-      <c r="V13" t="n">
-        <v>127</v>
-      </c>
       <c r="W13" t="n">
-        <v>386</v>
+        <v>397</v>
       </c>
       <c r="X13" t="n">
-        <v>475</v>
+        <v>499</v>
       </c>
       <c r="Y13" t="n">
-        <v>505</v>
+        <v>524</v>
       </c>
       <c r="Z13" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="AA13" t="n">
-        <v>1696</v>
+        <v>1770</v>
       </c>
       <c r="AB13" t="n">
-        <v>1999.72</v>
+        <v>2071.52</v>
       </c>
       <c r="AC13" t="n">
-        <v>1758.72</v>
+        <v>1824.52</v>
       </c>
       <c r="AD13" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>2225</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>202</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>449</v>
+      </c>
+      <c r="AH13" t="n">
+        <v>71</v>
+      </c>
+      <c r="AI13" t="n">
+        <v>243</v>
+      </c>
+      <c r="AJ13" t="n">
+        <v>140</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>254</v>
+      </c>
+      <c r="AL13" t="n">
+        <v>113</v>
+      </c>
+      <c r="AM13" t="n">
+        <v>300</v>
+      </c>
+      <c r="AN13" t="n">
+        <v>129</v>
+      </c>
+      <c r="AO13" t="n">
+        <v>77</v>
+      </c>
+      <c r="AP13" t="n">
+        <v>196</v>
+      </c>
+      <c r="AQ13" t="n">
+        <v>229</v>
+      </c>
+      <c r="AR13" t="n">
+        <v>239</v>
+      </c>
+      <c r="AS13" t="n">
+        <v>35</v>
+      </c>
+      <c r="AT13" t="n">
+        <v>999.7600000000001</v>
+      </c>
+      <c r="AU13" t="n">
+        <v>886.7600000000001</v>
+      </c>
+      <c r="AV13" t="n">
+        <v>0.7533543401955403</v>
+      </c>
+      <c r="AW13" t="n">
+        <v>0.8970354519330868</v>
+      </c>
+      <c r="AX13" t="n">
+        <v>84.79436881259511</v>
+      </c>
+      <c r="AY13" t="n">
+        <v>101.9322365993565</v>
+      </c>
+      <c r="AZ13" t="n">
+        <v>-17.1378677867614</v>
+      </c>
+      <c r="BA13" t="n">
+        <v>0.2771059079766087</v>
+      </c>
+      <c r="BB13" t="n">
+        <v>0.7035055059056577</v>
+      </c>
+      <c r="BC13" t="n">
+        <v>0.4931052979364868</v>
+      </c>
+      <c r="BD13" t="n">
+        <v>11</v>
+      </c>
+      <c r="BE13" t="n">
+        <v>2400</v>
+      </c>
+      <c r="BF13" t="n">
+        <v>216</v>
+      </c>
+      <c r="BG13" t="n">
+        <v>478</v>
+      </c>
+      <c r="BH13" t="n">
+        <v>66</v>
+      </c>
+      <c r="BI13" t="n">
+        <v>248</v>
+      </c>
+      <c r="BJ13" t="n">
+        <v>197</v>
+      </c>
+      <c r="BK13" t="n">
+        <v>329</v>
+      </c>
+      <c r="BL13" t="n">
+        <v>134</v>
+      </c>
+      <c r="BM13" t="n">
+        <v>369</v>
+      </c>
+      <c r="BN13" t="n">
+        <v>132</v>
+      </c>
+      <c r="BO13" t="n">
+        <v>54</v>
+      </c>
+      <c r="BP13" t="n">
+        <v>201</v>
+      </c>
+      <c r="BQ13" t="n">
+        <v>270</v>
+      </c>
+      <c r="BR13" t="n">
+        <v>285</v>
+      </c>
+      <c r="BS13" t="n">
+        <v>17</v>
+      </c>
+      <c r="BT13" t="n">
+        <v>1071.76</v>
+      </c>
+      <c r="BU13" t="n">
+        <v>937.76</v>
+      </c>
+      <c r="BV13" t="n">
+        <v>0.7695630161754164</v>
+      </c>
+      <c r="BW13" t="n">
+        <v>0.7811227857191141</v>
+      </c>
+      <c r="BX13" t="n">
+        <v>87.92439151574608</v>
+      </c>
+      <c r="BY13" t="n">
+        <v>89.13613750916981</v>
+      </c>
+      <c r="BZ13" t="n">
+        <v>-1.211745993423738</v>
+      </c>
+      <c r="CA13" t="n">
+        <v>0.3139505842966339</v>
+      </c>
+      <c r="CB13" t="n">
+        <v>0.7344160767033108</v>
+      </c>
+      <c r="CC13" t="n">
+        <v>0.5438953996471366</v>
+      </c>
+      <c r="CD13" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="14">
@@ -1744,88 +3876,244 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.8799761036781867</v>
+        <v>0.8823809761212461</v>
       </c>
       <c r="D14" t="n">
-        <v>0.8010601772164747</v>
+        <v>0.7971143611064209</v>
       </c>
       <c r="E14" t="n">
-        <v>102.0561002154936</v>
+        <v>102.2072859175755</v>
       </c>
       <c r="F14" t="n">
-        <v>90.04719660776537</v>
+        <v>89.50199670239273</v>
       </c>
       <c r="G14" t="n">
-        <v>12.00890360772826</v>
+        <v>12.70528921518279</v>
       </c>
       <c r="H14" t="n">
-        <v>0.3555718494602838</v>
+        <v>0.3501456486476293</v>
       </c>
       <c r="I14" t="n">
-        <v>0.7197637816016141</v>
+        <v>0.7240428266703186</v>
       </c>
       <c r="J14" t="n">
-        <v>0.5352791530150728</v>
+        <v>0.5337452767970261</v>
       </c>
       <c r="K14" t="n">
-        <v>4400</v>
+        <v>4600</v>
       </c>
       <c r="L14" t="n">
-        <v>1774</v>
+        <v>1848</v>
       </c>
       <c r="M14" t="n">
-        <v>430</v>
+        <v>443</v>
       </c>
       <c r="N14" t="n">
-        <v>887</v>
+        <v>916</v>
       </c>
       <c r="O14" t="n">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="P14" t="n">
-        <v>528</v>
+        <v>558</v>
       </c>
       <c r="Q14" t="n">
-        <v>416</v>
+        <v>431</v>
       </c>
       <c r="R14" t="n">
-        <v>621</v>
+        <v>644</v>
       </c>
       <c r="S14" t="n">
-        <v>284</v>
+        <v>293</v>
       </c>
       <c r="T14" t="n">
-        <v>543</v>
+        <v>570</v>
       </c>
       <c r="U14" t="n">
-        <v>340</v>
+        <v>353</v>
       </c>
       <c r="V14" t="n">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="W14" t="n">
-        <v>336</v>
+        <v>346</v>
       </c>
       <c r="X14" t="n">
-        <v>483</v>
+        <v>502</v>
       </c>
       <c r="Y14" t="n">
-        <v>513</v>
+        <v>537</v>
       </c>
       <c r="Z14" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AA14" t="n">
-        <v>1552</v>
+        <v>1603</v>
       </c>
       <c r="AB14" t="n">
-        <v>2024.24</v>
+        <v>2103.36</v>
       </c>
       <c r="AC14" t="n">
-        <v>1740.24</v>
+        <v>1810.36</v>
       </c>
       <c r="AD14" t="n">
-        <v>22</v>
+        <v>23</v>
+      </c>
+      <c r="AE14" t="n">
+        <v>2400</v>
+      </c>
+      <c r="AF14" t="n">
+        <v>227</v>
+      </c>
+      <c r="AG14" t="n">
+        <v>464</v>
+      </c>
+      <c r="AH14" t="n">
+        <v>87</v>
+      </c>
+      <c r="AI14" t="n">
+        <v>290</v>
+      </c>
+      <c r="AJ14" t="n">
+        <v>220</v>
+      </c>
+      <c r="AK14" t="n">
+        <v>330</v>
+      </c>
+      <c r="AL14" t="n">
+        <v>146</v>
+      </c>
+      <c r="AM14" t="n">
+        <v>281</v>
+      </c>
+      <c r="AN14" t="n">
+        <v>178</v>
+      </c>
+      <c r="AO14" t="n">
+        <v>122</v>
+      </c>
+      <c r="AP14" t="n">
+        <v>192</v>
+      </c>
+      <c r="AQ14" t="n">
+        <v>260</v>
+      </c>
+      <c r="AR14" t="n">
+        <v>275</v>
+      </c>
+      <c r="AS14" t="n">
+        <v>25</v>
+      </c>
+      <c r="AT14" t="n">
+        <v>1091.2</v>
+      </c>
+      <c r="AU14" t="n">
+        <v>945.2</v>
+      </c>
+      <c r="AV14" t="n">
+        <v>0.8579125355168932</v>
+      </c>
+      <c r="AW14" t="n">
+        <v>0.8001294364521695</v>
+      </c>
+      <c r="AX14" t="n">
+        <v>99.14644894654832</v>
+      </c>
+      <c r="AY14" t="n">
+        <v>90.47100931146706</v>
+      </c>
+      <c r="AZ14" t="n">
+        <v>8.675439635081265</v>
+      </c>
+      <c r="BA14" t="n">
+        <v>0.3391079582810658</v>
+      </c>
+      <c r="BB14" t="n">
+        <v>0.6987378860353025</v>
+      </c>
+      <c r="BC14" t="n">
+        <v>0.5115993662105542</v>
+      </c>
+      <c r="BD14" t="n">
+        <v>12</v>
+      </c>
+      <c r="BE14" t="n">
+        <v>2200</v>
+      </c>
+      <c r="BF14" t="n">
+        <v>216</v>
+      </c>
+      <c r="BG14" t="n">
+        <v>452</v>
+      </c>
+      <c r="BH14" t="n">
+        <v>90</v>
+      </c>
+      <c r="BI14" t="n">
+        <v>268</v>
+      </c>
+      <c r="BJ14" t="n">
+        <v>211</v>
+      </c>
+      <c r="BK14" t="n">
+        <v>314</v>
+      </c>
+      <c r="BL14" t="n">
+        <v>147</v>
+      </c>
+      <c r="BM14" t="n">
+        <v>289</v>
+      </c>
+      <c r="BN14" t="n">
+        <v>175</v>
+      </c>
+      <c r="BO14" t="n">
+        <v>101</v>
+      </c>
+      <c r="BP14" t="n">
+        <v>154</v>
+      </c>
+      <c r="BQ14" t="n">
+        <v>242</v>
+      </c>
+      <c r="BR14" t="n">
+        <v>262</v>
+      </c>
+      <c r="BS14" t="n">
+        <v>20</v>
+      </c>
+      <c r="BT14" t="n">
+        <v>1012.16</v>
+      </c>
+      <c r="BU14" t="n">
+        <v>865.16</v>
+      </c>
+      <c r="BV14" t="n">
+        <v>0.9090738204169039</v>
+      </c>
+      <c r="BW14" t="n">
+        <v>0.7938251880019677</v>
+      </c>
+      <c r="BX14" t="n">
+        <v>105.5463807950597</v>
+      </c>
+      <c r="BY14" t="n">
+        <v>88.44489203794801</v>
+      </c>
+      <c r="BZ14" t="n">
+        <v>17.10148875711173</v>
+      </c>
+      <c r="CA14" t="n">
+        <v>0.3621867654111532</v>
+      </c>
+      <c r="CB14" t="n">
+        <v>0.7516482164539725</v>
+      </c>
+      <c r="CC14" t="n">
+        <v>0.5579044519822681</v>
+      </c>
+      <c r="CD14" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="15">
@@ -1840,88 +4128,244 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.8853490855213964</v>
+        <v>0.880149129064686</v>
       </c>
       <c r="D15" t="n">
-        <v>0.8236939815713545</v>
+        <v>0.8256619498203585</v>
       </c>
       <c r="E15" t="n">
-        <v>100.4537761277143</v>
+        <v>100.0750519163378</v>
       </c>
       <c r="F15" t="n">
-        <v>93.65181179708325</v>
+        <v>93.68616920294927</v>
       </c>
       <c r="G15" t="n">
-        <v>6.801964330631065</v>
+        <v>6.388882713388553</v>
       </c>
       <c r="H15" t="n">
-        <v>0.3206387008983376</v>
+        <v>0.3273500617288446</v>
       </c>
       <c r="I15" t="n">
-        <v>0.7008047185347842</v>
+        <v>0.7044125039803929</v>
       </c>
       <c r="J15" t="n">
-        <v>0.513855830278152</v>
+        <v>0.518617603891129</v>
       </c>
       <c r="K15" t="n">
-        <v>4400</v>
+        <v>4600</v>
       </c>
       <c r="L15" t="n">
-        <v>1909</v>
+        <v>1997</v>
       </c>
       <c r="M15" t="n">
-        <v>504</v>
+        <v>534</v>
       </c>
       <c r="N15" t="n">
-        <v>984</v>
+        <v>1036</v>
       </c>
       <c r="O15" t="n">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="P15" t="n">
-        <v>558</v>
+        <v>582</v>
       </c>
       <c r="Q15" t="n">
-        <v>397</v>
+        <v>410</v>
       </c>
       <c r="R15" t="n">
-        <v>568</v>
+        <v>586</v>
       </c>
       <c r="S15" t="n">
-        <v>259</v>
+        <v>278</v>
       </c>
       <c r="T15" t="n">
-        <v>595</v>
+        <v>624</v>
       </c>
       <c r="U15" t="n">
-        <v>389</v>
+        <v>407</v>
       </c>
       <c r="V15" t="n">
+        <v>220</v>
+      </c>
+      <c r="W15" t="n">
+        <v>402</v>
+      </c>
+      <c r="X15" t="n">
+        <v>513</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>525</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>80</v>
+      </c>
+      <c r="AA15" t="n">
+        <v>1850</v>
+      </c>
+      <c r="AB15" t="n">
+        <v>2277.84</v>
+      </c>
+      <c r="AC15" t="n">
+        <v>1999.84</v>
+      </c>
+      <c r="AD15" t="n">
+        <v>23</v>
+      </c>
+      <c r="AE15" t="n">
+        <v>2200</v>
+      </c>
+      <c r="AF15" t="n">
+        <v>233</v>
+      </c>
+      <c r="AG15" t="n">
+        <v>482</v>
+      </c>
+      <c r="AH15" t="n">
+        <v>76</v>
+      </c>
+      <c r="AI15" t="n">
+        <v>273</v>
+      </c>
+      <c r="AJ15" t="n">
         <v>207</v>
       </c>
-      <c r="W15" t="n">
-        <v>371</v>
-      </c>
-      <c r="X15" t="n">
-        <v>494</v>
-      </c>
-      <c r="Y15" t="n">
-        <v>508</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>76</v>
-      </c>
-      <c r="AA15" t="n">
-        <v>1763</v>
-      </c>
-      <c r="AB15" t="n">
-        <v>2162.92</v>
-      </c>
-      <c r="AC15" t="n">
-        <v>1903.92</v>
-      </c>
-      <c r="AD15" t="n">
-        <v>22</v>
+      <c r="AK15" t="n">
+        <v>292</v>
+      </c>
+      <c r="AL15" t="n">
+        <v>128</v>
+      </c>
+      <c r="AM15" t="n">
+        <v>295</v>
+      </c>
+      <c r="AN15" t="n">
+        <v>167</v>
+      </c>
+      <c r="AO15" t="n">
+        <v>98</v>
+      </c>
+      <c r="AP15" t="n">
+        <v>188</v>
+      </c>
+      <c r="AQ15" t="n">
+        <v>252</v>
+      </c>
+      <c r="AR15" t="n">
+        <v>257</v>
+      </c>
+      <c r="AS15" t="n">
+        <v>44</v>
+      </c>
+      <c r="AT15" t="n">
+        <v>1071.48</v>
+      </c>
+      <c r="AU15" t="n">
+        <v>943.48</v>
+      </c>
+      <c r="AV15" t="n">
+        <v>0.8417005746116856</v>
+      </c>
+      <c r="AW15" t="n">
+        <v>0.8470073855075468</v>
+      </c>
+      <c r="AX15" t="n">
+        <v>95.58730700069906</v>
+      </c>
+      <c r="AY15" t="n">
+        <v>95.04760365974967</v>
+      </c>
+      <c r="AZ15" t="n">
+        <v>0.5397033409494014</v>
+      </c>
+      <c r="BA15" t="n">
+        <v>0.3078753317739781</v>
+      </c>
+      <c r="BB15" t="n">
+        <v>0.7223581563243425</v>
+      </c>
+      <c r="BC15" t="n">
+        <v>0.5121215224769812</v>
+      </c>
+      <c r="BD15" t="n">
+        <v>11</v>
+      </c>
+      <c r="BE15" t="n">
+        <v>2400</v>
+      </c>
+      <c r="BF15" t="n">
+        <v>301</v>
+      </c>
+      <c r="BG15" t="n">
+        <v>554</v>
+      </c>
+      <c r="BH15" t="n">
+        <v>97</v>
+      </c>
+      <c r="BI15" t="n">
+        <v>309</v>
+      </c>
+      <c r="BJ15" t="n">
+        <v>203</v>
+      </c>
+      <c r="BK15" t="n">
+        <v>294</v>
+      </c>
+      <c r="BL15" t="n">
+        <v>150</v>
+      </c>
+      <c r="BM15" t="n">
+        <v>329</v>
+      </c>
+      <c r="BN15" t="n">
+        <v>240</v>
+      </c>
+      <c r="BO15" t="n">
+        <v>122</v>
+      </c>
+      <c r="BP15" t="n">
+        <v>214</v>
+      </c>
+      <c r="BQ15" t="n">
+        <v>261</v>
+      </c>
+      <c r="BR15" t="n">
+        <v>268</v>
+      </c>
+      <c r="BS15" t="n">
+        <v>36</v>
+      </c>
+      <c r="BT15" t="n">
+        <v>1206.36</v>
+      </c>
+      <c r="BU15" t="n">
+        <v>1056.36</v>
+      </c>
+      <c r="BV15" t="n">
+        <v>0.9153936373132697</v>
+      </c>
+      <c r="BW15" t="n">
+        <v>0.8060953004404361</v>
+      </c>
+      <c r="BX15" t="n">
+        <v>104.1888180890067</v>
+      </c>
+      <c r="BY15" t="n">
+        <v>92.43818761754891</v>
+      </c>
+      <c r="BZ15" t="n">
+        <v>11.75063047145778</v>
+      </c>
+      <c r="CA15" t="n">
+        <v>0.3452018975208058</v>
+      </c>
+      <c r="CB15" t="n">
+        <v>0.6879623226651059</v>
+      </c>
+      <c r="CC15" t="n">
+        <v>0.5245723451874311</v>
+      </c>
+      <c r="CD15" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>